<commit_message>
feat(cuchi): deploy Cu Chi Tunnels Pillar Travel Guide with UNESCO 2026 data, 3-column magazine layout, and verified internal links
</commit_message>
<xml_diff>
--- a/KE_HOACH_25_BAI_VIET_CU_CHI_SEO_GEO.xlsx
+++ b/KE_HOACH_25_BAI_VIET_CU_CHI_SEO_GEO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huynhtronghieu/Documents/thericetour/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E2817F9-AF3B-E446-9BCC-23BBA66D5039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E28B46-E8BA-7B45-8AB8-3C0B75716BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1580" windowWidth="30240" windowHeight="13440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="25_Bai_Viet_Cu_Chi_Matrix" sheetId="1" r:id="rId1"/>
@@ -1158,7 +1158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1179,9 +1179,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1644,208 +1641,208 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:13" s="23" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="11" t="s">
+      <c r="J3" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="K3" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="L3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="18" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:13" s="23" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="24" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:13" s="23" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="I5" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J5" s="11" t="s">
+      <c r="J5" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="K5" s="10" t="s">
+      <c r="K5" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="L5" s="7" t="s">
+      <c r="L5" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M5" s="7" t="s">
+      <c r="M5" s="18" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:13" s="24" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="25" t="s">
+    <row r="6" spans="1:13" s="23" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="E6" s="27" t="s">
+      <c r="E6" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="F6" s="29" t="s">
+      <c r="F6" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="G6" s="29" t="s">
+      <c r="G6" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="H6" s="29" t="s">
+      <c r="H6" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="I6" s="28" t="s">
+      <c r="I6" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="29" t="s">
+      <c r="J6" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="K6" s="28" t="s">
+      <c r="K6" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="L6" s="25" t="s">
+      <c r="L6" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="M6" s="25" t="s">
+      <c r="M6" s="24" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="24" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="19" t="s">
+    <row r="7" spans="1:13" s="23" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="E7" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="H7" s="23" t="s">
+      <c r="H7" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="I7" s="22" t="s">
+      <c r="I7" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="23" t="s">
+      <c r="J7" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="K7" s="22" t="s">
+      <c r="K7" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="L7" s="19" t="s">
+      <c r="L7" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M7" s="19" t="s">
+      <c r="M7" s="18" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1897,31 +1894,31 @@
       <c r="B9" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="I9" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J9" s="11" t="s">
+      <c r="J9" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="K9" s="9" t="s">
         <v>61</v>
       </c>
       <c r="L9" s="7" t="s">
@@ -1979,31 +1976,31 @@
       <c r="B11" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="H11" s="11" t="s">
+      <c r="H11" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="11" t="s">
+      <c r="J11" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="K11" s="10" t="s">
+      <c r="K11" s="9" t="s">
         <v>61</v>
       </c>
       <c r="L11" s="7" t="s">
@@ -2061,31 +2058,31 @@
       <c r="B13" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="H13" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="I13" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="J13" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="K13" s="10" t="s">
+      <c r="K13" s="9" t="s">
         <v>61</v>
       </c>
       <c r="L13" s="7" t="s">
@@ -2143,31 +2140,31 @@
       <c r="B15" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="H15" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="I15" s="10" t="s">
+      <c r="I15" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="J15" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="K15" s="10" t="s">
+      <c r="K15" s="9" t="s">
         <v>61</v>
       </c>
       <c r="L15" s="7" t="s">
@@ -2225,31 +2222,31 @@
       <c r="B17" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="G17" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="H17" s="11" t="s">
+      <c r="H17" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="I17" s="10" t="s">
+      <c r="I17" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J17" s="11" t="s">
+      <c r="J17" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="K17" s="10" t="s">
+      <c r="K17" s="9" t="s">
         <v>61</v>
       </c>
       <c r="L17" s="7" t="s">
@@ -2307,31 +2304,31 @@
       <c r="B19" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G19" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="H19" s="11" t="s">
+      <c r="H19" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="I19" s="10" t="s">
+      <c r="I19" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J19" s="11" t="s">
+      <c r="J19" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="K19" s="10" t="s">
+      <c r="K19" s="9" t="s">
         <v>61</v>
       </c>
       <c r="L19" s="7" t="s">
@@ -2389,31 +2386,31 @@
       <c r="B21" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="F21" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="G21" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="H21" s="11" t="s">
+      <c r="H21" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="I21" s="10" t="s">
+      <c r="I21" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J21" s="11" t="s">
+      <c r="J21" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="K21" s="10" t="s">
+      <c r="K21" s="9" t="s">
         <v>61</v>
       </c>
       <c r="L21" s="7" t="s">
@@ -2471,31 +2468,31 @@
       <c r="B23" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="F23" s="11" t="s">
+      <c r="F23" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="G23" s="11" t="s">
+      <c r="G23" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="H23" s="11" t="s">
+      <c r="H23" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="I23" s="10" t="s">
+      <c r="I23" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J23" s="11" t="s">
+      <c r="J23" s="10" t="s">
         <v>204</v>
       </c>
-      <c r="K23" s="10" t="s">
+      <c r="K23" s="9" t="s">
         <v>205</v>
       </c>
       <c r="L23" s="7" t="s">
@@ -2550,34 +2547,34 @@
       <c r="A25" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="11" t="s">
         <v>215</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="F25" s="11" t="s">
+      <c r="F25" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="G25" s="11" t="s">
+      <c r="G25" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="H25" s="11" t="s">
+      <c r="H25" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="I25" s="10" t="s">
+      <c r="I25" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J25" s="11" t="s">
+      <c r="J25" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="K25" s="10" t="s">
+      <c r="K25" s="9" t="s">
         <v>223</v>
       </c>
       <c r="L25" s="7" t="s">
@@ -2591,7 +2588,7 @@
       <c r="A26" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="12" t="s">
         <v>215</v>
       </c>
       <c r="C26" s="4" t="s">
@@ -2697,22 +2694,22 @@
       <c r="A3" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>245</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="13" t="s">
         <v>250</v>
       </c>
     </row>
@@ -2735,7 +2732,7 @@
       <c r="F4" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="14" t="s">
         <v>255</v>
       </c>
     </row>
@@ -2743,22 +2740,22 @@
       <c r="A5" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>256</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="13" t="s">
         <v>255</v>
       </c>
     </row>
@@ -2778,28 +2775,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>260</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>261</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="15" t="s">
         <v>262</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="15" t="s">
         <v>263</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="15" t="s">
         <v>264</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="15" t="s">
         <v>265</v>
       </c>
     </row>
@@ -2821,19 +2818,19 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>271</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>275</v>
       </c>
     </row>
@@ -2855,19 +2852,19 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="8" t="s">
         <v>281</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="10" t="s">
         <v>285</v>
       </c>
     </row>
@@ -2889,19 +2886,19 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="10" t="s">
         <v>295</v>
       </c>
     </row>
@@ -2923,28 +2920,28 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="16" t="s">
         <v>301</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
     </row>
     <row r="13" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="15" t="s">
         <v>302</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="15" t="s">
         <v>303</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="15" t="s">
         <v>304</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="15" t="s">
         <v>305</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="15" t="s">
         <v>306</v>
       </c>
     </row>
@@ -2966,19 +2963,19 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="10" t="s">
         <v>315</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="10" t="s">
         <v>316</v>
       </c>
     </row>
@@ -3000,19 +2997,19 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="8" t="s">
         <v>320</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="10" t="s">
         <v>322</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="10" t="s">
         <v>323</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="10" t="s">
         <v>324</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(cuchi): publish How Far Are The Cu Chi Tunnels From Ho Chi Minh City with verified transit logistics, UNESCO 2026 data, and 3-column magazine layout
</commit_message>
<xml_diff>
--- a/KE_HOACH_25_BAI_VIET_CU_CHI_SEO_GEO.xlsx
+++ b/KE_HOACH_25_BAI_VIET_CU_CHI_SEO_GEO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huynhtronghieu/Documents/thericetour/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E28B46-E8BA-7B45-8AB8-3C0B75716BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E3A3099-E0EA-6D42-938F-D52F716DC81B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1580" windowWidth="30240" windowHeight="13440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,20 @@
     <sheet name="Lo_Trinh_Sprint_Gantt" sheetId="2" r:id="rId2"/>
     <sheet name="Cu_Chi_Fact_Base" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1600,44 +1613,44 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:13" s="23" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="24" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
perf(d1): optimize db queries, add edge caching, bot filtering and performance indexes
</commit_message>
<xml_diff>
--- a/KE_HOACH_25_BAI_VIET_CU_CHI_SEO_GEO.xlsx
+++ b/KE_HOACH_25_BAI_VIET_CU_CHI_SEO_GEO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huynhtronghieu/Documents/thericetour/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E3A3099-E0EA-6D42-938F-D52F716DC81B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF0A66C-AAFA-D64E-9213-3D5E9A214598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1580" windowWidth="30240" windowHeight="13440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1859,44 +1859,44 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:13" s="23" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J8" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="K8" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="M8" s="24" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1982,44 +1982,44 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+    <row r="11" spans="1:13" s="23" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="10" t="s">
+      <c r="J11" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="L11" s="7" t="s">
+      <c r="L11" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="M11" s="7" t="s">
+      <c r="M11" s="18" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>